<commit_message>
docs: add UC specs
complete UC specs are UC02-UC19
add skeleton specs for UC19-UC32
</commit_message>
<xml_diff>
--- a/Project Binder/Planning/Gantt Chart.xlsx
+++ b/Project Binder/Planning/Gantt Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nexus\Documents\GitHub\csg-in2033\Project Binder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\csg-in2033\Project Binder\Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2C56154-DACB-42B7-A798-391D158B9F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8D93696-FED8-4514-B06B-451904B18BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-93" yWindow="-93" windowWidth="20666" windowHeight="12266" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project schedule" sheetId="11" r:id="rId1"/>
@@ -167,7 +167,7 @@
     <numFmt numFmtId="166" formatCode="ddd\,\ m/d/yyyy"/>
     <numFmt numFmtId="167" formatCode="mmm\ d\,\ yyyy"/>
     <numFmt numFmtId="168" formatCode="d"/>
-    <numFmt numFmtId="170" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="169" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="26" x14ac:knownFonts="1">
     <font>
@@ -869,6 +869,64 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="169" fontId="15" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="3" borderId="6" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="3" borderId="7" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="4" borderId="5" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="5" borderId="8" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="23" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -880,64 +938,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="23" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="15" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="15" fillId="3" borderId="6" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="15" fillId="3" borderId="7" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="15" fillId="4" borderId="5" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="15" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="15" fillId="5" borderId="8" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -1460,20 +1460,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BL33"/>
-  <sheetFormatPr defaultColWidth="8.71875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.71875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="22.71875" customWidth="1"/>
-    <col min="3" max="3" width="16.71875" customWidth="1"/>
-    <col min="4" max="4" width="10.71875" customWidth="1"/>
-    <col min="5" max="5" width="10.71875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.71875" customWidth="1"/>
-    <col min="7" max="7" width="2.71875" customWidth="1"/>
+    <col min="1" max="1" width="2.75" style="7" customWidth="1"/>
+    <col min="2" max="2" width="22.75" customWidth="1"/>
+    <col min="3" max="3" width="16.75" customWidth="1"/>
+    <col min="4" max="4" width="10.75" customWidth="1"/>
+    <col min="5" max="5" width="10.75" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.75" customWidth="1"/>
+    <col min="7" max="7" width="2.75" customWidth="1"/>
     <col min="8" max="8" width="6" hidden="1" customWidth="1"/>
-    <col min="9" max="65" width="2.71875" customWidth="1"/>
+    <col min="9" max="65" width="2.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" ht="90" customHeight="1" x14ac:dyDescent="2.5">
+    <row r="1" spans="1:64" ht="90" customHeight="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A1" s="8"/>
       <c r="B1" s="71" t="s">
         <v>10</v>
@@ -1483,30 +1483,30 @@
       <c r="E1" s="14"/>
       <c r="F1" s="15"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="80" t="s">
+      <c r="I1" s="92" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="81"/>
-      <c r="M1" s="81"/>
-      <c r="N1" s="81"/>
-      <c r="O1" s="81"/>
+      <c r="J1" s="93"/>
+      <c r="K1" s="93"/>
+      <c r="L1" s="93"/>
+      <c r="M1" s="93"/>
+      <c r="N1" s="93"/>
+      <c r="O1" s="93"/>
       <c r="P1" s="17"/>
-      <c r="Q1" s="85">
+      <c r="Q1" s="90">
         <v>46048</v>
       </c>
-      <c r="R1" s="86"/>
-      <c r="S1" s="86"/>
-      <c r="T1" s="86"/>
-      <c r="U1" s="86"/>
-      <c r="V1" s="86"/>
-      <c r="W1" s="86"/>
-      <c r="X1" s="86"/>
-      <c r="Y1" s="86"/>
-      <c r="Z1" s="86"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="91"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
     </row>
-    <row r="2" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="1.05">
+    <row r="2" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B2" s="69" t="s">
         <v>11</v>
       </c>
@@ -1514,135 +1514,135 @@
         <v>12</v>
       </c>
       <c r="F2" s="16"/>
-      <c r="I2" s="80" t="s">
+      <c r="I2" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="81"/>
-      <c r="K2" s="81"/>
-      <c r="L2" s="81"/>
-      <c r="M2" s="81"/>
-      <c r="N2" s="81"/>
-      <c r="O2" s="81"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="93"/>
+      <c r="L2" s="93"/>
+      <c r="M2" s="93"/>
+      <c r="N2" s="93"/>
+      <c r="O2" s="93"/>
       <c r="P2" s="17"/>
-      <c r="Q2" s="78">
+      <c r="Q2" s="88">
         <v>1</v>
       </c>
-      <c r="R2" s="79"/>
-      <c r="S2" s="79"/>
-      <c r="T2" s="79"/>
-      <c r="U2" s="79"/>
-      <c r="V2" s="79"/>
-      <c r="W2" s="79"/>
-      <c r="X2" s="79"/>
-      <c r="Y2" s="79"/>
-      <c r="Z2" s="79"/>
+      <c r="R2" s="89"/>
+      <c r="S2" s="89"/>
+      <c r="T2" s="89"/>
+      <c r="U2" s="89"/>
+      <c r="V2" s="89"/>
+      <c r="W2" s="89"/>
+      <c r="X2" s="89"/>
+      <c r="Y2" s="89"/>
+      <c r="Z2" s="89"/>
     </row>
-    <row r="3" spans="1:64" s="19" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:64" s="19" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="18"/>
       <c r="D3" s="20"/>
       <c r="E3" s="21"/>
     </row>
-    <row r="4" spans="1:64" s="19" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:64" s="19" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="8"/>
       <c r="B4" s="22"/>
       <c r="E4" s="23"/>
-      <c r="I4" s="84">
+      <c r="I4" s="85">
         <f>I5</f>
         <v>46048</v>
       </c>
-      <c r="J4" s="82"/>
-      <c r="K4" s="82"/>
-      <c r="L4" s="82"/>
-      <c r="M4" s="82"/>
-      <c r="N4" s="82"/>
-      <c r="O4" s="82"/>
-      <c r="P4" s="82">
+      <c r="J4" s="83"/>
+      <c r="K4" s="83"/>
+      <c r="L4" s="83"/>
+      <c r="M4" s="83"/>
+      <c r="N4" s="83"/>
+      <c r="O4" s="83"/>
+      <c r="P4" s="83">
         <f>P5</f>
         <v>46055</v>
       </c>
-      <c r="Q4" s="82"/>
-      <c r="R4" s="82"/>
-      <c r="S4" s="82"/>
-      <c r="T4" s="82"/>
-      <c r="U4" s="82"/>
-      <c r="V4" s="82"/>
-      <c r="W4" s="82">
+      <c r="Q4" s="83"/>
+      <c r="R4" s="83"/>
+      <c r="S4" s="83"/>
+      <c r="T4" s="83"/>
+      <c r="U4" s="83"/>
+      <c r="V4" s="83"/>
+      <c r="W4" s="83">
         <f>W5</f>
         <v>46062</v>
       </c>
-      <c r="X4" s="82"/>
-      <c r="Y4" s="82"/>
-      <c r="Z4" s="82"/>
-      <c r="AA4" s="82"/>
-      <c r="AB4" s="82"/>
-      <c r="AC4" s="82"/>
-      <c r="AD4" s="82">
+      <c r="X4" s="83"/>
+      <c r="Y4" s="83"/>
+      <c r="Z4" s="83"/>
+      <c r="AA4" s="83"/>
+      <c r="AB4" s="83"/>
+      <c r="AC4" s="83"/>
+      <c r="AD4" s="83">
         <f>AD5</f>
         <v>46069</v>
       </c>
-      <c r="AE4" s="82"/>
-      <c r="AF4" s="82"/>
-      <c r="AG4" s="82"/>
-      <c r="AH4" s="82"/>
-      <c r="AI4" s="82"/>
-      <c r="AJ4" s="82"/>
-      <c r="AK4" s="82">
+      <c r="AE4" s="83"/>
+      <c r="AF4" s="83"/>
+      <c r="AG4" s="83"/>
+      <c r="AH4" s="83"/>
+      <c r="AI4" s="83"/>
+      <c r="AJ4" s="83"/>
+      <c r="AK4" s="83">
         <f>AK5</f>
         <v>46076</v>
       </c>
-      <c r="AL4" s="82"/>
-      <c r="AM4" s="82"/>
-      <c r="AN4" s="82"/>
-      <c r="AO4" s="82"/>
-      <c r="AP4" s="82"/>
-      <c r="AQ4" s="82"/>
-      <c r="AR4" s="82">
+      <c r="AL4" s="83"/>
+      <c r="AM4" s="83"/>
+      <c r="AN4" s="83"/>
+      <c r="AO4" s="83"/>
+      <c r="AP4" s="83"/>
+      <c r="AQ4" s="83"/>
+      <c r="AR4" s="83">
         <f>AR5</f>
         <v>46083</v>
       </c>
-      <c r="AS4" s="82"/>
-      <c r="AT4" s="82"/>
-      <c r="AU4" s="82"/>
-      <c r="AV4" s="82"/>
-      <c r="AW4" s="82"/>
-      <c r="AX4" s="82"/>
-      <c r="AY4" s="82">
+      <c r="AS4" s="83"/>
+      <c r="AT4" s="83"/>
+      <c r="AU4" s="83"/>
+      <c r="AV4" s="83"/>
+      <c r="AW4" s="83"/>
+      <c r="AX4" s="83"/>
+      <c r="AY4" s="83">
         <f>AY5</f>
         <v>46090</v>
       </c>
-      <c r="AZ4" s="82"/>
-      <c r="BA4" s="82"/>
-      <c r="BB4" s="82"/>
-      <c r="BC4" s="82"/>
-      <c r="BD4" s="82"/>
-      <c r="BE4" s="82"/>
-      <c r="BF4" s="82">
+      <c r="AZ4" s="83"/>
+      <c r="BA4" s="83"/>
+      <c r="BB4" s="83"/>
+      <c r="BC4" s="83"/>
+      <c r="BD4" s="83"/>
+      <c r="BE4" s="83"/>
+      <c r="BF4" s="83">
         <f>BF5</f>
         <v>46097</v>
       </c>
-      <c r="BG4" s="82"/>
-      <c r="BH4" s="82"/>
-      <c r="BI4" s="82"/>
-      <c r="BJ4" s="82"/>
-      <c r="BK4" s="82"/>
-      <c r="BL4" s="83"/>
+      <c r="BG4" s="83"/>
+      <c r="BH4" s="83"/>
+      <c r="BI4" s="83"/>
+      <c r="BJ4" s="83"/>
+      <c r="BK4" s="83"/>
+      <c r="BL4" s="84"/>
     </row>
-    <row r="5" spans="1:64" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="72"/>
-      <c r="B5" s="73" t="s">
+    <row r="5" spans="1:64" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="94"/>
+      <c r="B5" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="75" t="s">
+      <c r="C5" s="97" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="77" t="s">
+      <c r="D5" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="77" t="s">
+      <c r="E5" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="77" t="s">
+      <c r="F5" s="86" t="s">
         <v>3</v>
       </c>
       <c r="I5" s="24">
@@ -1870,13 +1870,13 @@
         <v>46103</v>
       </c>
     </row>
-    <row r="6" spans="1:64" s="19" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="72"/>
-      <c r="B6" s="74"/>
-      <c r="C6" s="76"/>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-      <c r="F6" s="76"/>
+    <row r="6" spans="1:64" s="19" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="94"/>
+      <c r="B6" s="96"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
+      <c r="E6" s="87"/>
+      <c r="F6" s="87"/>
       <c r="I6" s="27" t="str">
         <f t="shared" ref="I6:AN6" si="3">LEFT(TEXT(I5,"ddd"),1)</f>
         <v>M</v>
@@ -2102,7 +2102,7 @@
         <v>S</v>
       </c>
     </row>
-    <row r="7" spans="1:64" s="19" customFormat="1" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:64" s="19" customFormat="1" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>5</v>
       </c>
@@ -2172,15 +2172,15 @@
       <c r="BK7" s="32"/>
       <c r="BL7" s="32"/>
     </row>
-    <row r="8" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="33" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="34"/>
       <c r="D8" s="35"/>
-      <c r="E8" s="87"/>
-      <c r="F8" s="88"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="73"/>
       <c r="G8" s="11"/>
       <c r="H8" s="5" t="str">
         <f t="shared" ref="H8:H30" si="5">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -2243,7 +2243,7 @@
       <c r="BK8" s="36"/>
       <c r="BL8" s="36"/>
     </row>
-    <row r="9" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="38" t="s">
         <v>15</v>
@@ -2254,10 +2254,10 @@
       <c r="D9" s="40">
         <v>1</v>
       </c>
-      <c r="E9" s="89">
+      <c r="E9" s="74">
         <v>46055</v>
       </c>
-      <c r="F9" s="89">
+      <c r="F9" s="74">
         <v>46055</v>
       </c>
       <c r="G9" s="11"/>
@@ -2322,7 +2322,7 @@
       <c r="BK9" s="41"/>
       <c r="BL9" s="41"/>
     </row>
-    <row r="10" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="42" t="s">
         <v>17</v>
@@ -2333,10 +2333,10 @@
       <c r="D10" s="44">
         <v>0.33</v>
       </c>
-      <c r="E10" s="90">
+      <c r="E10" s="75">
         <v>46048</v>
       </c>
-      <c r="F10" s="90">
+      <c r="F10" s="75">
         <v>46061</v>
       </c>
       <c r="G10" s="11"/>
@@ -2401,7 +2401,7 @@
       <c r="BK10" s="41"/>
       <c r="BL10" s="41"/>
     </row>
-    <row r="11" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
       <c r="B11" s="42" t="s">
         <v>19</v>
@@ -2412,10 +2412,10 @@
       <c r="D11" s="44">
         <v>1</v>
       </c>
-      <c r="E11" s="90">
+      <c r="E11" s="75">
         <v>46056</v>
       </c>
-      <c r="F11" s="90">
+      <c r="F11" s="75">
         <v>46056</v>
       </c>
       <c r="G11" s="11"/>
@@ -2480,22 +2480,22 @@
       <c r="BK11" s="41"/>
       <c r="BL11" s="41"/>
     </row>
-    <row r="12" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="46" t="s">
         <v>13</v>
       </c>
       <c r="C12" s="47"/>
       <c r="D12" s="48"/>
-      <c r="E12" s="91"/>
-      <c r="F12" s="92"/>
+      <c r="E12" s="76"/>
+      <c r="F12" s="77"/>
       <c r="G12" s="11"/>
       <c r="H12" s="5" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="49" t="s">
         <v>21</v>
@@ -2504,8 +2504,8 @@
         <v>31</v>
       </c>
       <c r="D13" s="51"/>
-      <c r="E13" s="93"/>
-      <c r="F13" s="93"/>
+      <c r="E13" s="78"/>
+      <c r="F13" s="78"/>
       <c r="G13" s="11"/>
       <c r="H13" s="5" t="str">
         <f t="shared" si="5"/>
@@ -2568,7 +2568,7 @@
       <c r="BK13" s="41"/>
       <c r="BL13" s="41"/>
     </row>
-    <row r="14" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="49" t="s">
         <v>22</v>
@@ -2577,8 +2577,8 @@
         <v>32</v>
       </c>
       <c r="D14" s="51"/>
-      <c r="E14" s="93"/>
-      <c r="F14" s="93"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="78"/>
       <c r="G14" s="11"/>
       <c r="H14" s="5" t="str">
         <f t="shared" si="5"/>
@@ -2641,7 +2641,7 @@
       <c r="BK14" s="41"/>
       <c r="BL14" s="41"/>
     </row>
-    <row r="15" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
       <c r="B15" s="49" t="s">
         <v>23</v>
@@ -2649,13 +2649,19 @@
       <c r="C15" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="51"/>
-      <c r="E15" s="93"/>
-      <c r="F15" s="93"/>
+      <c r="D15" s="51">
+        <v>0.59</v>
+      </c>
+      <c r="E15" s="78">
+        <v>46058</v>
+      </c>
+      <c r="F15" s="78">
+        <v>46065</v>
+      </c>
       <c r="G15" s="11"/>
-      <c r="H15" s="5" t="str">
+      <c r="H15" s="5">
         <f t="shared" si="5"/>
-        <v/>
+        <v>8</v>
       </c>
       <c r="I15" s="41"/>
       <c r="J15" s="41"/>
@@ -2714,17 +2720,17 @@
       <c r="BK15" s="41"/>
       <c r="BL15" s="41"/>
     </row>
-    <row r="16" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
-      <c r="B16" s="97" t="s">
+      <c r="B16" s="82" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="51"/>
-      <c r="E16" s="93"/>
-      <c r="F16" s="93"/>
+      <c r="E16" s="78"/>
+      <c r="F16" s="78"/>
       <c r="G16" s="11"/>
       <c r="H16" s="5" t="str">
         <f t="shared" si="5"/>
@@ -2787,17 +2793,17 @@
       <c r="BK16" s="41"/>
       <c r="BL16" s="41"/>
     </row>
-    <row r="17" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
-      <c r="B17" s="97" t="s">
+      <c r="B17" s="82" t="s">
         <v>24</v>
       </c>
       <c r="C17" s="50" t="s">
         <v>34</v>
       </c>
       <c r="D17" s="51"/>
-      <c r="E17" s="93"/>
-      <c r="F17" s="93"/>
+      <c r="E17" s="78"/>
+      <c r="F17" s="78"/>
       <c r="G17" s="11"/>
       <c r="H17" s="5" t="str">
         <f t="shared" si="5"/>
@@ -2860,15 +2866,15 @@
       <c r="BK17" s="41"/>
       <c r="BL17" s="41"/>
     </row>
-    <row r="18" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
-      <c r="B18" s="97" t="s">
+      <c r="B18" s="82" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="97"/>
-      <c r="D18" s="97"/>
-      <c r="E18" s="97"/>
-      <c r="F18" s="97"/>
+      <c r="C18" s="82"/>
+      <c r="D18" s="82"/>
+      <c r="E18" s="82"/>
+      <c r="F18" s="82"/>
       <c r="G18" s="11"/>
       <c r="H18" s="5"/>
       <c r="I18" s="41"/>
@@ -2928,15 +2934,15 @@
       <c r="BK18" s="41"/>
       <c r="BL18" s="41"/>
     </row>
-    <row r="19" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
-      <c r="B19" s="97" t="s">
+      <c r="B19" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="97"/>
-      <c r="D19" s="97"/>
-      <c r="E19" s="97"/>
-      <c r="F19" s="97"/>
+      <c r="C19" s="82"/>
+      <c r="D19" s="82"/>
+      <c r="E19" s="82"/>
+      <c r="F19" s="82"/>
       <c r="G19" s="11"/>
       <c r="H19" s="5"/>
       <c r="I19" s="55"/>
@@ -2996,15 +3002,15 @@
       <c r="BK19" s="55"/>
       <c r="BL19" s="55"/>
     </row>
-    <row r="20" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
-      <c r="B20" s="97" t="s">
+      <c r="B20" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="97"/>
-      <c r="D20" s="97"/>
-      <c r="E20" s="97"/>
-      <c r="F20" s="97"/>
+      <c r="C20" s="82"/>
+      <c r="D20" s="82"/>
+      <c r="E20" s="82"/>
+      <c r="F20" s="82"/>
       <c r="G20" s="11"/>
       <c r="H20" s="5"/>
       <c r="I20" s="55"/>
@@ -3064,17 +3070,17 @@
       <c r="BK20" s="55"/>
       <c r="BL20" s="55"/>
     </row>
-    <row r="21" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="97" t="s">
+      <c r="B21" s="82" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="97" t="s">
+      <c r="C21" s="82" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="97"/>
-      <c r="E21" s="97"/>
-      <c r="F21" s="97"/>
+      <c r="D21" s="82"/>
+      <c r="E21" s="82"/>
+      <c r="F21" s="82"/>
       <c r="G21" s="11"/>
       <c r="H21" s="5"/>
       <c r="I21" s="55"/>
@@ -3134,15 +3140,15 @@
       <c r="BK21" s="55"/>
       <c r="BL21" s="55"/>
     </row>
-    <row r="22" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="97" t="s">
+      <c r="B22" s="82" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="97"/>
-      <c r="D22" s="97"/>
-      <c r="E22" s="97"/>
-      <c r="F22" s="97"/>
+      <c r="C22" s="82"/>
+      <c r="D22" s="82"/>
+      <c r="E22" s="82"/>
+      <c r="F22" s="82"/>
       <c r="G22" s="11"/>
       <c r="H22" s="5"/>
       <c r="I22" s="55"/>
@@ -3202,15 +3208,15 @@
       <c r="BK22" s="55"/>
       <c r="BL22" s="55"/>
     </row>
-    <row r="23" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
       <c r="B23" s="52" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="53"/>
       <c r="D23" s="54"/>
-      <c r="E23" s="94"/>
-      <c r="F23" s="95"/>
+      <c r="E23" s="79"/>
+      <c r="F23" s="80"/>
       <c r="G23" s="11"/>
       <c r="H23" s="5" t="str">
         <f t="shared" si="5"/>
@@ -3273,13 +3279,13 @@
       <c r="BK23" s="55"/>
       <c r="BL23" s="55"/>
     </row>
-    <row r="24" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
       <c r="B24" s="56"/>
       <c r="C24" s="57"/>
       <c r="D24" s="58"/>
-      <c r="E24" s="96"/>
-      <c r="F24" s="96"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="81"/>
       <c r="G24" s="11"/>
       <c r="H24" s="5" t="str">
         <f t="shared" si="5"/>
@@ -3342,13 +3348,13 @@
       <c r="BK24" s="41"/>
       <c r="BL24" s="41"/>
     </row>
-    <row r="25" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
       <c r="B25" s="56"/>
       <c r="C25" s="57"/>
       <c r="D25" s="58"/>
-      <c r="E25" s="96"/>
-      <c r="F25" s="96"/>
+      <c r="E25" s="81"/>
+      <c r="F25" s="81"/>
       <c r="G25" s="11"/>
       <c r="H25" s="5" t="str">
         <f t="shared" si="5"/>
@@ -3411,13 +3417,13 @@
       <c r="BK25" s="41"/>
       <c r="BL25" s="41"/>
     </row>
-    <row r="26" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
       <c r="B26" s="56"/>
       <c r="C26" s="57"/>
       <c r="D26" s="58"/>
-      <c r="E26" s="96"/>
-      <c r="F26" s="96"/>
+      <c r="E26" s="81"/>
+      <c r="F26" s="81"/>
       <c r="G26" s="11"/>
       <c r="H26" s="5" t="str">
         <f t="shared" si="5"/>
@@ -3480,13 +3486,13 @@
       <c r="BK26" s="41"/>
       <c r="BL26" s="41"/>
     </row>
-    <row r="27" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" s="56"/>
       <c r="C27" s="57"/>
       <c r="D27" s="58"/>
-      <c r="E27" s="96"/>
-      <c r="F27" s="96"/>
+      <c r="E27" s="81"/>
+      <c r="F27" s="81"/>
       <c r="G27" s="11"/>
       <c r="H27" s="5" t="str">
         <f t="shared" si="5"/>
@@ -3549,13 +3555,13 @@
       <c r="BK27" s="41"/>
       <c r="BL27" s="41"/>
     </row>
-    <row r="28" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" s="56"/>
       <c r="C28" s="57"/>
       <c r="D28" s="58"/>
-      <c r="E28" s="96"/>
-      <c r="F28" s="96"/>
+      <c r="E28" s="81"/>
+      <c r="F28" s="81"/>
       <c r="G28" s="11"/>
       <c r="H28" s="5" t="str">
         <f t="shared" si="5"/>
@@ -3618,7 +3624,7 @@
       <c r="BK28" s="41"/>
       <c r="BL28" s="41"/>
     </row>
-    <row r="29" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" s="59"/>
       <c r="C29" s="60"/>
@@ -3687,7 +3693,7 @@
       <c r="BK29" s="36"/>
       <c r="BL29" s="36"/>
     </row>
-    <row r="30" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:64" s="37" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8"/>
       <c r="B30" s="63" t="s">
         <v>0</v>
@@ -3758,18 +3764,28 @@
       <c r="BK30" s="68"/>
       <c r="BL30" s="68"/>
     </row>
-    <row r="31" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G31" s="3"/>
     </row>
-    <row r="32" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="10"/>
       <c r="F32" s="9"/>
     </row>
-    <row r="33" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C33" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="Q2:Z2"/>
+    <mergeCell ref="Q1:Z1"/>
+    <mergeCell ref="I1:O1"/>
+    <mergeCell ref="I2:O2"/>
     <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
@@ -3778,16 +3794,6 @@
     <mergeCell ref="AK4:AQ4"/>
     <mergeCell ref="AR4:AX4"/>
     <mergeCell ref="AY4:BE4"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="Q2:Z2"/>
-    <mergeCell ref="Q1:Z1"/>
-    <mergeCell ref="I1:O1"/>
-    <mergeCell ref="I2:O2"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D17 D23:D30">
     <cfRule type="dataBar" priority="23">
@@ -3899,15 +3905,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4219,6 +4216,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
   <ds:schemaRefs>
@@ -4239,14 +4245,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A09426A3-87E9-4865-8A6C-3456B026AE03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4267,6 +4265,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>